<commit_message>
Scan plans: draw basic single-V weld scan plans and print them on the weld report
New Scan plans pages (list, edit with a live drawing, fill from a setup)
draw the weld, wedge at the index offset and the sectorial beam fan with
Pillow. A weld report can pick a scan plan; it prints on a Scan Plan page
at the end of the Excel report, both sides side by side.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel_templates/paut_weld.xlsx
+++ b/excel_templates/paut_weld.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MistrasFHR-PB2\Desktop\Coding\PAUT-Workflow-Automation\excel_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4324EA34-8B0D-42DD-A00F-9CB4A6DCA3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2CC49C8-26A5-4B21-99E5-96DF15F2C5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="769" xr2:uid="{C7A2BE69-112F-4BDE-9DBC-04CBA0DD1E9B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="769" xr2:uid="{C7A2BE69-112F-4BDE-9DBC-04CBA0DD1E9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="5" r:id="rId1"/>
     <sheet name="Indication" sheetId="7" r:id="rId2"/>
     <sheet name="Continuation" sheetId="11" r:id="rId3"/>
+    <sheet name="Scan Plan" sheetId="25" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="142">
   <si>
     <t>Date</t>
   </si>
@@ -413,6 +414,9 @@
   </si>
   <si>
     <t>Exam Code/Specification</t>
+  </si>
+  <si>
+    <t>Scan Plan</t>
   </si>
   <si>
     <t>100-UTFORM-010 rev 1.3</t>
@@ -464,6 +468,9 @@
   </si>
   <si>
     <t>Reviewed By:</t>
+  </si>
+  <si>
+    <t>Pipe Size</t>
   </si>
 </sst>
 </file>
@@ -2337,7 +2344,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="443">
+  <cellXfs count="449">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -3792,6 +3799,24 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -4260,6 +4285,139 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>155575</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3409950" cy="744238"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DBFACCCD-A6FD-45B2-9F2B-6D89DE8DD9D1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5889625" y="1"/>
+          <a:ext cx="3409950" cy="744238"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" rtlCol="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Phased Array Examination</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> Report</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1800" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>511969</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0431920-ED85-432B-ADB3-25ADA357C392}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:srcRect r="26436"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="276225" y="9525"/>
+          <a:ext cx="3207544" cy="600075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -4608,7 +4766,7 @@
       </c>
       <c r="W1" s="146"/>
       <c r="X1" s="147" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Y1" s="147"/>
       <c r="Z1" s="147"/>
@@ -4949,7 +5107,7 @@
     </row>
     <row r="13" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="268" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B13" s="140"/>
       <c r="C13" s="140"/>
@@ -4958,34 +5116,34 @@
         <v>12</v>
       </c>
       <c r="F13" s="271" t="s">
+        <v>132</v>
+      </c>
+      <c r="G13" s="271" t="s">
+        <v>133</v>
+      </c>
+      <c r="H13" s="271" t="s">
         <v>131</v>
       </c>
-      <c r="G13" s="271" t="s">
-        <v>132</v>
-      </c>
-      <c r="H13" s="271" t="s">
-        <v>130</v>
-      </c>
       <c r="I13" s="273" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J13" s="139" t="s">
         <v>1</v>
       </c>
       <c r="K13" s="161"/>
       <c r="L13" s="268" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M13" s="277"/>
       <c r="N13" s="268" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="O13" s="277"/>
       <c r="P13" s="295" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Q13" s="273" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="R13" s="297"/>
       <c r="S13" s="273" t="s">
@@ -4993,7 +5151,7 @@
       </c>
       <c r="T13" s="299"/>
       <c r="U13" s="276" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="V13" s="277"/>
       <c r="W13" s="280" t="s">
@@ -5364,7 +5522,7 @@
       <c r="H24" s="80"/>
       <c r="I24" s="81"/>
       <c r="J24" s="100" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K24" s="101"/>
       <c r="L24" s="104"/>
@@ -5531,7 +5689,7 @@
       <c r="C29" s="98"/>
       <c r="D29" s="99"/>
       <c r="E29" s="67" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F29" s="79"/>
       <c r="G29" s="80"/>
@@ -5565,7 +5723,7 @@
       <c r="C30" s="98"/>
       <c r="D30" s="99"/>
       <c r="E30" s="67" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F30" s="79"/>
       <c r="G30" s="80"/>
@@ -6429,7 +6587,7 @@
     </row>
     <row r="57" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="120" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B57" s="121"/>
       <c r="C57" s="172"/>
@@ -7091,7 +7249,7 @@
         <v>42</v>
       </c>
       <c r="W2" s="146"/>
-      <c r="X2" s="434" t="str">
+      <c r="X2" s="440" t="str">
         <f>IF(Report!X2="","",Report!X2)</f>
         <v/>
       </c>
@@ -7228,7 +7386,7 @@
         <v>51</v>
       </c>
       <c r="B7" s="160"/>
-      <c r="C7" s="435" t="str">
+      <c r="C7" s="441" t="str">
         <f>IF(Report!C7="","",Report!C7)</f>
         <v/>
       </c>
@@ -7261,7 +7419,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="101"/>
-      <c r="C8" s="436" t="str">
+      <c r="C8" s="442" t="str">
         <f>IF(Report!C8="","",Report!C8)</f>
         <v/>
       </c>
@@ -7294,7 +7452,7 @@
         <v>65</v>
       </c>
       <c r="B9" s="101"/>
-      <c r="C9" s="436" t="str">
+      <c r="C9" s="442" t="str">
         <f>IF(Report!C9="","",Report!C9)</f>
         <v/>
       </c>
@@ -7327,7 +7485,7 @@
         <v>58</v>
       </c>
       <c r="B10" s="101"/>
-      <c r="C10" s="436" t="str">
+      <c r="C10" s="442" t="str">
         <f>IF(Report!C10="","",Report!C10)</f>
         <v/>
       </c>
@@ -7360,7 +7518,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="101"/>
-      <c r="C11" s="436" t="str">
+      <c r="C11" s="442" t="str">
         <f>IF(Report!C11="","",Report!C11)</f>
         <v/>
       </c>
@@ -7374,7 +7532,7 @@
         <v>31</v>
       </c>
       <c r="K11" s="370"/>
-      <c r="L11" s="437" t="str">
+      <c r="L11" s="443" t="str">
         <f>IF(Report!L11="","",Report!L11)</f>
         <v/>
       </c>
@@ -7388,7 +7546,7 @@
         <v>11</v>
       </c>
       <c r="T11" s="370"/>
-      <c r="U11" s="437" t="str">
+      <c r="U11" s="443" t="str">
         <f>IF(Report!U11="","",Report!U11)</f>
         <v/>
       </c>
@@ -7398,7 +7556,7 @@
       <c r="Y11" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="Z11" s="438" t="str">
+      <c r="Z11" s="444" t="str">
         <f>IF(Report!Z11="","",Report!Z11)</f>
         <v/>
       </c>
@@ -8872,7 +9030,7 @@
         <v>44</v>
       </c>
       <c r="B64" s="121"/>
-      <c r="C64" s="439" t="str">
+      <c r="C64" s="445" t="str">
         <f>IF(Report!C55="","",Report!C55)</f>
         <v/>
       </c>
@@ -8887,7 +9045,7 @@
       <c r="J64" s="395"/>
       <c r="K64" s="395"/>
       <c r="L64" s="395"/>
-      <c r="M64" s="440" t="str">
+      <c r="M64" s="446" t="str">
         <f>IF(Report!R55="","",Report!R55)</f>
         <v/>
       </c>
@@ -9244,7 +9402,7 @@
         <v>51</v>
       </c>
       <c r="B7" s="160"/>
-      <c r="C7" s="435" t="str">
+      <c r="C7" s="441" t="str">
         <f>IF(Report!C7="","",Report!C7)</f>
         <v/>
       </c>
@@ -9277,7 +9435,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="101"/>
-      <c r="C8" s="436" t="str">
+      <c r="C8" s="442" t="str">
         <f>IF(Report!C8="","",Report!C8)</f>
         <v/>
       </c>
@@ -9310,7 +9468,7 @@
         <v>65</v>
       </c>
       <c r="B9" s="101"/>
-      <c r="C9" s="436" t="str">
+      <c r="C9" s="442" t="str">
         <f>IF(Report!C9="","",Report!C9)</f>
         <v/>
       </c>
@@ -9343,7 +9501,7 @@
         <v>58</v>
       </c>
       <c r="B10" s="101"/>
-      <c r="C10" s="436" t="str">
+      <c r="C10" s="442" t="str">
         <f>IF(Report!C10="","",Report!C10)</f>
         <v/>
       </c>
@@ -9376,7 +9534,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="95"/>
-      <c r="C11" s="436" t="str">
+      <c r="C11" s="442" t="str">
         <f>IF(Report!C11="","",Report!C11)</f>
         <v/>
       </c>
@@ -9390,7 +9548,7 @@
         <v>31</v>
       </c>
       <c r="K11" s="95"/>
-      <c r="L11" s="437" t="str">
+      <c r="L11" s="443" t="str">
         <f>IF(Report!L11="","",Report!L11)</f>
         <v/>
       </c>
@@ -9404,7 +9562,7 @@
         <v>11</v>
       </c>
       <c r="T11" s="95"/>
-      <c r="U11" s="437" t="str">
+      <c r="U11" s="443" t="str">
         <f>IF(Report!U11="","",Report!U11)</f>
         <v/>
       </c>
@@ -9414,7 +9572,7 @@
       <c r="Y11" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="Z11" s="438" t="str">
+      <c r="Z11" s="444" t="str">
         <f>IF(Report!Z11="","",Report!Z11)</f>
         <v/>
       </c>
@@ -10590,7 +10748,7 @@
         <v>44</v>
       </c>
       <c r="B52" s="121"/>
-      <c r="C52" s="441" t="str">
+      <c r="C52" s="447" t="str">
         <f>IF(Report!C55="","",Report!C55)</f>
         <v/>
       </c>
@@ -10603,7 +10761,7 @@
       </c>
       <c r="I52" s="380"/>
       <c r="J52" s="380"/>
-      <c r="K52" s="442" t="str">
+      <c r="K52" s="448" t="str">
         <f>IF(Report!R55="","",Report!R55)</f>
         <v/>
       </c>
@@ -10842,6 +11000,2020 @@
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C
 </oddFooter>
+  </headerFooter>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B524E67-D9D9-4BCF-8C63-BC31BC9EAFEA}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:Z66"/>
+  <sheetFormatPr defaultColWidth="5.7109375" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" style="1"/>
+    <col min="2" max="2" width="12.85546875" style="1" customWidth="1"/>
+    <col min="3" max="4" width="6.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12" style="1" customWidth="1"/>
+    <col min="12" max="12" width="5.7109375" style="1" customWidth="1"/>
+    <col min="13" max="15" width="4.85546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="9.7109375" style="1" customWidth="1"/>
+    <col min="17" max="18" width="4.5703125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="5.7109375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="4.85546875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="5.7109375" style="1"/>
+    <col min="22" max="22" width="10.42578125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="5.7109375" style="1"/>
+    <col min="24" max="24" width="7" style="1" customWidth="1"/>
+    <col min="25" max="25" width="5.7109375" style="1" customWidth="1"/>
+    <col min="26" max="26" width="11.7109375" style="1" customWidth="1"/>
+    <col min="27" max="27" width="5.7109375" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="5.7109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" ht="12" x14ac:dyDescent="0.2">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="146" t="s">
+        <v>70</v>
+      </c>
+      <c r="W1" s="146"/>
+      <c r="X1" s="433" t="str">
+        <f>IF(Report!X1="","",Report!X1)</f>
+        <v>100-UTFORM-010 rev 1.3</v>
+      </c>
+      <c r="Y1" s="358"/>
+      <c r="Z1" s="358"/>
+    </row>
+    <row r="2" spans="1:26" ht="12" x14ac:dyDescent="0.2">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="V2" s="146" t="s">
+        <v>42</v>
+      </c>
+      <c r="W2" s="146"/>
+      <c r="X2" s="440" t="str">
+        <f>IF(Report!X2="","",Report!X2)</f>
+        <v/>
+      </c>
+      <c r="Y2" s="359"/>
+      <c r="Z2" s="359"/>
+    </row>
+    <row r="3" spans="1:26" ht="12" x14ac:dyDescent="0.2">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="V3" s="146" t="s">
+        <v>40</v>
+      </c>
+      <c r="W3" s="146"/>
+      <c r="X3" s="360" t="str">
+        <f>IF(Report!X3="","",Report!X3)</f>
+        <v/>
+      </c>
+      <c r="Y3" s="361"/>
+      <c r="Z3" s="361"/>
+    </row>
+    <row r="4" spans="1:26" ht="12" x14ac:dyDescent="0.2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="V4" s="146" t="s">
+        <v>78</v>
+      </c>
+      <c r="W4" s="146"/>
+      <c r="X4" s="41"/>
+      <c r="Y4" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z4" s="41"/>
+    </row>
+    <row r="5" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="V5" s="245" t="s">
+        <v>79</v>
+      </c>
+      <c r="W5" s="245"/>
+      <c r="X5" s="362" t="str">
+        <f>IF(Report!X5="","",Report!X5)</f>
+        <v/>
+      </c>
+      <c r="Y5" s="363"/>
+      <c r="Z5" s="363"/>
+    </row>
+    <row r="6" spans="1:26" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="152" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="153"/>
+      <c r="C6" s="153"/>
+      <c r="D6" s="153"/>
+      <c r="E6" s="153"/>
+      <c r="F6" s="153"/>
+      <c r="G6" s="153"/>
+      <c r="H6" s="153"/>
+      <c r="I6" s="153"/>
+      <c r="J6" s="153"/>
+      <c r="K6" s="153"/>
+      <c r="L6" s="153"/>
+      <c r="M6" s="153"/>
+      <c r="N6" s="153"/>
+      <c r="O6" s="153"/>
+      <c r="P6" s="153"/>
+      <c r="Q6" s="153"/>
+      <c r="R6" s="153"/>
+      <c r="S6" s="153"/>
+      <c r="T6" s="153"/>
+      <c r="U6" s="153"/>
+      <c r="V6" s="153"/>
+      <c r="W6" s="153"/>
+      <c r="X6" s="153"/>
+      <c r="Y6" s="153"/>
+      <c r="Z6" s="154"/>
+    </row>
+    <row r="7" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="159" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="160"/>
+      <c r="C7" s="441" t="str">
+        <f>IF(Report!C7="","",Report!C7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="364"/>
+      <c r="E7" s="364"/>
+      <c r="F7" s="364"/>
+      <c r="G7" s="364"/>
+      <c r="H7" s="364"/>
+      <c r="I7" s="364"/>
+      <c r="J7" s="364"/>
+      <c r="K7" s="364"/>
+      <c r="L7" s="364"/>
+      <c r="M7" s="364"/>
+      <c r="N7" s="364"/>
+      <c r="O7" s="364"/>
+      <c r="P7" s="364"/>
+      <c r="Q7" s="364"/>
+      <c r="R7" s="364"/>
+      <c r="S7" s="364"/>
+      <c r="T7" s="364"/>
+      <c r="U7" s="364"/>
+      <c r="V7" s="364"/>
+      <c r="W7" s="364"/>
+      <c r="X7" s="364"/>
+      <c r="Y7" s="364"/>
+      <c r="Z7" s="365"/>
+    </row>
+    <row r="8" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="100" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="101"/>
+      <c r="C8" s="442" t="str">
+        <f>IF(Report!C8="","",Report!C8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="366"/>
+      <c r="E8" s="366"/>
+      <c r="F8" s="366"/>
+      <c r="G8" s="366"/>
+      <c r="H8" s="366"/>
+      <c r="I8" s="366"/>
+      <c r="J8" s="366"/>
+      <c r="K8" s="366"/>
+      <c r="L8" s="366"/>
+      <c r="M8" s="366"/>
+      <c r="N8" s="366"/>
+      <c r="O8" s="366"/>
+      <c r="P8" s="366"/>
+      <c r="Q8" s="366"/>
+      <c r="R8" s="366"/>
+      <c r="S8" s="366"/>
+      <c r="T8" s="366"/>
+      <c r="U8" s="366"/>
+      <c r="V8" s="366"/>
+      <c r="W8" s="366"/>
+      <c r="X8" s="366"/>
+      <c r="Y8" s="366"/>
+      <c r="Z8" s="367"/>
+    </row>
+    <row r="9" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="100" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="101"/>
+      <c r="C9" s="442" t="str">
+        <f>IF(Report!C9="","",Report!C9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="366"/>
+      <c r="E9" s="366"/>
+      <c r="F9" s="366"/>
+      <c r="G9" s="366"/>
+      <c r="H9" s="366"/>
+      <c r="I9" s="366"/>
+      <c r="J9" s="366"/>
+      <c r="K9" s="366"/>
+      <c r="L9" s="366"/>
+      <c r="M9" s="366"/>
+      <c r="N9" s="366"/>
+      <c r="O9" s="366"/>
+      <c r="P9" s="366"/>
+      <c r="Q9" s="366"/>
+      <c r="R9" s="366"/>
+      <c r="S9" s="366"/>
+      <c r="T9" s="366"/>
+      <c r="U9" s="366"/>
+      <c r="V9" s="366"/>
+      <c r="W9" s="366"/>
+      <c r="X9" s="366"/>
+      <c r="Y9" s="366"/>
+      <c r="Z9" s="367"/>
+    </row>
+    <row r="10" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="100" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="101"/>
+      <c r="C10" s="442" t="str">
+        <f>IF(Report!C10="","",Report!C10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="366"/>
+      <c r="E10" s="366"/>
+      <c r="F10" s="366"/>
+      <c r="G10" s="366"/>
+      <c r="H10" s="366"/>
+      <c r="I10" s="366"/>
+      <c r="J10" s="366"/>
+      <c r="K10" s="366"/>
+      <c r="L10" s="366"/>
+      <c r="M10" s="366"/>
+      <c r="N10" s="366"/>
+      <c r="O10" s="366"/>
+      <c r="P10" s="366"/>
+      <c r="Q10" s="366"/>
+      <c r="R10" s="366"/>
+      <c r="S10" s="366"/>
+      <c r="T10" s="366"/>
+      <c r="U10" s="366"/>
+      <c r="V10" s="366"/>
+      <c r="W10" s="366"/>
+      <c r="X10" s="366"/>
+      <c r="Y10" s="366"/>
+      <c r="Z10" s="367"/>
+    </row>
+    <row r="11" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="100" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="101"/>
+      <c r="C11" s="442" t="str">
+        <f>IF(Report!C11="","",Report!C11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="366"/>
+      <c r="E11" s="366"/>
+      <c r="F11" s="366"/>
+      <c r="G11" s="366"/>
+      <c r="H11" s="366"/>
+      <c r="I11" s="368"/>
+      <c r="J11" s="369" t="s">
+        <v>31</v>
+      </c>
+      <c r="K11" s="370"/>
+      <c r="L11" s="443" t="str">
+        <f>IF(Report!L11="","",Report!L11)</f>
+        <v/>
+      </c>
+      <c r="M11" s="371"/>
+      <c r="N11" s="371"/>
+      <c r="O11" s="371"/>
+      <c r="P11" s="371"/>
+      <c r="Q11" s="371"/>
+      <c r="R11" s="372"/>
+      <c r="S11" s="369" t="s">
+        <v>11</v>
+      </c>
+      <c r="T11" s="370"/>
+      <c r="U11" s="443" t="str">
+        <f>IF(Report!U11="","",Report!U11)</f>
+        <v/>
+      </c>
+      <c r="V11" s="102"/>
+      <c r="W11" s="102"/>
+      <c r="X11" s="169"/>
+      <c r="Y11" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z11" s="444" t="str">
+        <f>IF(Report!Z11="","",Report!Z11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="434"/>
+      <c r="B12" s="435"/>
+      <c r="C12" s="435"/>
+      <c r="D12" s="435"/>
+      <c r="E12" s="435"/>
+      <c r="F12" s="435"/>
+      <c r="G12" s="435"/>
+      <c r="H12" s="435"/>
+      <c r="I12" s="435"/>
+      <c r="J12" s="435"/>
+      <c r="K12" s="435"/>
+      <c r="L12" s="435"/>
+      <c r="M12" s="435"/>
+      <c r="N12" s="435"/>
+      <c r="O12" s="435"/>
+      <c r="P12" s="435"/>
+      <c r="Q12" s="435"/>
+      <c r="R12" s="435"/>
+      <c r="S12" s="435"/>
+      <c r="T12" s="435"/>
+      <c r="U12" s="435"/>
+      <c r="V12" s="435"/>
+      <c r="W12" s="435"/>
+      <c r="X12" s="435"/>
+      <c r="Y12" s="435"/>
+      <c r="Z12" s="436"/>
+    </row>
+    <row r="13" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="437"/>
+      <c r="B13" s="438"/>
+      <c r="C13" s="438"/>
+      <c r="D13" s="438"/>
+      <c r="E13" s="438"/>
+      <c r="F13" s="438"/>
+      <c r="G13" s="438"/>
+      <c r="H13" s="438"/>
+      <c r="I13" s="438"/>
+      <c r="J13" s="438"/>
+      <c r="K13" s="438"/>
+      <c r="L13" s="438"/>
+      <c r="M13" s="438"/>
+      <c r="N13" s="438"/>
+      <c r="O13" s="438"/>
+      <c r="P13" s="438"/>
+      <c r="Q13" s="438"/>
+      <c r="R13" s="438"/>
+      <c r="S13" s="438"/>
+      <c r="T13" s="438"/>
+      <c r="U13" s="438"/>
+      <c r="V13" s="438"/>
+      <c r="W13" s="438"/>
+      <c r="X13" s="438"/>
+      <c r="Y13" s="438"/>
+      <c r="Z13" s="439"/>
+    </row>
+    <row r="14" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="437"/>
+      <c r="B14" s="438"/>
+      <c r="C14" s="438"/>
+      <c r="D14" s="438"/>
+      <c r="E14" s="438"/>
+      <c r="F14" s="438"/>
+      <c r="G14" s="438"/>
+      <c r="H14" s="438"/>
+      <c r="I14" s="438"/>
+      <c r="J14" s="438"/>
+      <c r="K14" s="438"/>
+      <c r="L14" s="438"/>
+      <c r="M14" s="438"/>
+      <c r="N14" s="438"/>
+      <c r="O14" s="438"/>
+      <c r="P14" s="438"/>
+      <c r="Q14" s="438"/>
+      <c r="R14" s="438"/>
+      <c r="S14" s="438"/>
+      <c r="T14" s="438"/>
+      <c r="U14" s="438"/>
+      <c r="V14" s="438"/>
+      <c r="W14" s="438"/>
+      <c r="X14" s="438"/>
+      <c r="Y14" s="438"/>
+      <c r="Z14" s="439"/>
+    </row>
+    <row r="15" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="437"/>
+      <c r="B15" s="438"/>
+      <c r="C15" s="438"/>
+      <c r="D15" s="438"/>
+      <c r="E15" s="438"/>
+      <c r="F15" s="438"/>
+      <c r="G15" s="438"/>
+      <c r="H15" s="438"/>
+      <c r="I15" s="438"/>
+      <c r="J15" s="438"/>
+      <c r="K15" s="438"/>
+      <c r="L15" s="438"/>
+      <c r="M15" s="438"/>
+      <c r="N15" s="438"/>
+      <c r="O15" s="438"/>
+      <c r="P15" s="438"/>
+      <c r="Q15" s="438"/>
+      <c r="R15" s="438"/>
+      <c r="S15" s="438"/>
+      <c r="T15" s="438"/>
+      <c r="U15" s="438"/>
+      <c r="V15" s="438"/>
+      <c r="W15" s="438"/>
+      <c r="X15" s="438"/>
+      <c r="Y15" s="438"/>
+      <c r="Z15" s="439"/>
+    </row>
+    <row r="16" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="437"/>
+      <c r="B16" s="438"/>
+      <c r="C16" s="438"/>
+      <c r="D16" s="438"/>
+      <c r="E16" s="438"/>
+      <c r="F16" s="438"/>
+      <c r="G16" s="438"/>
+      <c r="H16" s="438"/>
+      <c r="I16" s="438"/>
+      <c r="J16" s="438"/>
+      <c r="K16" s="438"/>
+      <c r="L16" s="438"/>
+      <c r="M16" s="438"/>
+      <c r="N16" s="438"/>
+      <c r="O16" s="438"/>
+      <c r="P16" s="438"/>
+      <c r="Q16" s="438"/>
+      <c r="R16" s="438"/>
+      <c r="S16" s="438"/>
+      <c r="T16" s="438"/>
+      <c r="U16" s="438"/>
+      <c r="V16" s="438"/>
+      <c r="W16" s="438"/>
+      <c r="X16" s="438"/>
+      <c r="Y16" s="438"/>
+      <c r="Z16" s="439"/>
+    </row>
+    <row r="17" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="437"/>
+      <c r="B17" s="438"/>
+      <c r="C17" s="438"/>
+      <c r="D17" s="438"/>
+      <c r="E17" s="438"/>
+      <c r="F17" s="438"/>
+      <c r="G17" s="438"/>
+      <c r="H17" s="438"/>
+      <c r="I17" s="438"/>
+      <c r="J17" s="438"/>
+      <c r="K17" s="438"/>
+      <c r="L17" s="438"/>
+      <c r="M17" s="438"/>
+      <c r="N17" s="438"/>
+      <c r="O17" s="438"/>
+      <c r="P17" s="438"/>
+      <c r="Q17" s="438"/>
+      <c r="R17" s="438"/>
+      <c r="S17" s="438"/>
+      <c r="T17" s="438"/>
+      <c r="U17" s="438"/>
+      <c r="V17" s="438"/>
+      <c r="W17" s="438"/>
+      <c r="X17" s="438"/>
+      <c r="Y17" s="438"/>
+      <c r="Z17" s="439"/>
+    </row>
+    <row r="18" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="437"/>
+      <c r="B18" s="438"/>
+      <c r="C18" s="438"/>
+      <c r="D18" s="438"/>
+      <c r="E18" s="438"/>
+      <c r="F18" s="438"/>
+      <c r="G18" s="438"/>
+      <c r="H18" s="438"/>
+      <c r="I18" s="438"/>
+      <c r="J18" s="438"/>
+      <c r="K18" s="438"/>
+      <c r="L18" s="438"/>
+      <c r="M18" s="438"/>
+      <c r="N18" s="438"/>
+      <c r="O18" s="438"/>
+      <c r="P18" s="438"/>
+      <c r="Q18" s="438"/>
+      <c r="R18" s="438"/>
+      <c r="S18" s="438"/>
+      <c r="T18" s="438"/>
+      <c r="U18" s="438"/>
+      <c r="V18" s="438"/>
+      <c r="W18" s="438"/>
+      <c r="X18" s="438"/>
+      <c r="Y18" s="438"/>
+      <c r="Z18" s="439"/>
+    </row>
+    <row r="19" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="437"/>
+      <c r="B19" s="438"/>
+      <c r="C19" s="438"/>
+      <c r="D19" s="438"/>
+      <c r="E19" s="438"/>
+      <c r="F19" s="438"/>
+      <c r="G19" s="438"/>
+      <c r="H19" s="438"/>
+      <c r="I19" s="438"/>
+      <c r="J19" s="438"/>
+      <c r="K19" s="438"/>
+      <c r="L19" s="438"/>
+      <c r="M19" s="438"/>
+      <c r="N19" s="438"/>
+      <c r="O19" s="438"/>
+      <c r="P19" s="438"/>
+      <c r="Q19" s="438"/>
+      <c r="R19" s="438"/>
+      <c r="S19" s="438"/>
+      <c r="T19" s="438"/>
+      <c r="U19" s="438"/>
+      <c r="V19" s="438"/>
+      <c r="W19" s="438"/>
+      <c r="X19" s="438"/>
+      <c r="Y19" s="438"/>
+      <c r="Z19" s="439"/>
+    </row>
+    <row r="20" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="437"/>
+      <c r="B20" s="438"/>
+      <c r="C20" s="438"/>
+      <c r="D20" s="438"/>
+      <c r="E20" s="438"/>
+      <c r="F20" s="438"/>
+      <c r="G20" s="438"/>
+      <c r="H20" s="438"/>
+      <c r="I20" s="438"/>
+      <c r="J20" s="438"/>
+      <c r="K20" s="438"/>
+      <c r="L20" s="438"/>
+      <c r="M20" s="438"/>
+      <c r="N20" s="438"/>
+      <c r="O20" s="438"/>
+      <c r="P20" s="438"/>
+      <c r="Q20" s="438"/>
+      <c r="R20" s="438"/>
+      <c r="S20" s="438"/>
+      <c r="T20" s="438"/>
+      <c r="U20" s="438"/>
+      <c r="V20" s="438"/>
+      <c r="W20" s="438"/>
+      <c r="X20" s="438"/>
+      <c r="Y20" s="438"/>
+      <c r="Z20" s="439"/>
+    </row>
+    <row r="21" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="437"/>
+      <c r="B21" s="438"/>
+      <c r="C21" s="438"/>
+      <c r="D21" s="438"/>
+      <c r="E21" s="438"/>
+      <c r="F21" s="438"/>
+      <c r="G21" s="438"/>
+      <c r="H21" s="438"/>
+      <c r="I21" s="438"/>
+      <c r="J21" s="438"/>
+      <c r="K21" s="438"/>
+      <c r="L21" s="438"/>
+      <c r="M21" s="438"/>
+      <c r="N21" s="438"/>
+      <c r="O21" s="438"/>
+      <c r="P21" s="438"/>
+      <c r="Q21" s="438"/>
+      <c r="R21" s="438"/>
+      <c r="S21" s="438"/>
+      <c r="T21" s="438"/>
+      <c r="U21" s="438"/>
+      <c r="V21" s="438"/>
+      <c r="W21" s="438"/>
+      <c r="X21" s="438"/>
+      <c r="Y21" s="438"/>
+      <c r="Z21" s="439"/>
+    </row>
+    <row r="22" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="437"/>
+      <c r="B22" s="438"/>
+      <c r="C22" s="438"/>
+      <c r="D22" s="438"/>
+      <c r="E22" s="438"/>
+      <c r="F22" s="438"/>
+      <c r="G22" s="438"/>
+      <c r="H22" s="438"/>
+      <c r="I22" s="438"/>
+      <c r="J22" s="438"/>
+      <c r="K22" s="438"/>
+      <c r="L22" s="438"/>
+      <c r="M22" s="438"/>
+      <c r="N22" s="438"/>
+      <c r="O22" s="438"/>
+      <c r="P22" s="438"/>
+      <c r="Q22" s="438"/>
+      <c r="R22" s="438"/>
+      <c r="S22" s="438"/>
+      <c r="T22" s="438"/>
+      <c r="U22" s="438"/>
+      <c r="V22" s="438"/>
+      <c r="W22" s="438"/>
+      <c r="X22" s="438"/>
+      <c r="Y22" s="438"/>
+      <c r="Z22" s="439"/>
+    </row>
+    <row r="23" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="437"/>
+      <c r="B23" s="438"/>
+      <c r="C23" s="438"/>
+      <c r="D23" s="438"/>
+      <c r="E23" s="438"/>
+      <c r="F23" s="438"/>
+      <c r="G23" s="438"/>
+      <c r="H23" s="438"/>
+      <c r="I23" s="438"/>
+      <c r="J23" s="438"/>
+      <c r="K23" s="438"/>
+      <c r="L23" s="438"/>
+      <c r="M23" s="438"/>
+      <c r="N23" s="438"/>
+      <c r="O23" s="438"/>
+      <c r="P23" s="438"/>
+      <c r="Q23" s="438"/>
+      <c r="R23" s="438"/>
+      <c r="S23" s="438"/>
+      <c r="T23" s="438"/>
+      <c r="U23" s="438"/>
+      <c r="V23" s="438"/>
+      <c r="W23" s="438"/>
+      <c r="X23" s="438"/>
+      <c r="Y23" s="438"/>
+      <c r="Z23" s="439"/>
+    </row>
+    <row r="24" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="437"/>
+      <c r="B24" s="438"/>
+      <c r="C24" s="438"/>
+      <c r="D24" s="438"/>
+      <c r="E24" s="438"/>
+      <c r="F24" s="438"/>
+      <c r="G24" s="438"/>
+      <c r="H24" s="438"/>
+      <c r="I24" s="438"/>
+      <c r="J24" s="438"/>
+      <c r="K24" s="438"/>
+      <c r="L24" s="438"/>
+      <c r="M24" s="438"/>
+      <c r="N24" s="438"/>
+      <c r="O24" s="438"/>
+      <c r="P24" s="438"/>
+      <c r="Q24" s="438"/>
+      <c r="R24" s="438"/>
+      <c r="S24" s="438"/>
+      <c r="T24" s="438"/>
+      <c r="U24" s="438"/>
+      <c r="V24" s="438"/>
+      <c r="W24" s="438"/>
+      <c r="X24" s="438"/>
+      <c r="Y24" s="438"/>
+      <c r="Z24" s="439"/>
+    </row>
+    <row r="25" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="437"/>
+      <c r="B25" s="438"/>
+      <c r="C25" s="438"/>
+      <c r="D25" s="438"/>
+      <c r="E25" s="438"/>
+      <c r="F25" s="438"/>
+      <c r="G25" s="438"/>
+      <c r="H25" s="438"/>
+      <c r="I25" s="438"/>
+      <c r="J25" s="438"/>
+      <c r="K25" s="438"/>
+      <c r="L25" s="438"/>
+      <c r="M25" s="438"/>
+      <c r="N25" s="438"/>
+      <c r="O25" s="438"/>
+      <c r="P25" s="438"/>
+      <c r="Q25" s="438"/>
+      <c r="R25" s="438"/>
+      <c r="S25" s="438"/>
+      <c r="T25" s="438"/>
+      <c r="U25" s="438"/>
+      <c r="V25" s="438"/>
+      <c r="W25" s="438"/>
+      <c r="X25" s="438"/>
+      <c r="Y25" s="438"/>
+      <c r="Z25" s="439"/>
+    </row>
+    <row r="26" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="437"/>
+      <c r="B26" s="438"/>
+      <c r="C26" s="438"/>
+      <c r="D26" s="438"/>
+      <c r="E26" s="438"/>
+      <c r="F26" s="438"/>
+      <c r="G26" s="438"/>
+      <c r="H26" s="438"/>
+      <c r="I26" s="438"/>
+      <c r="J26" s="438"/>
+      <c r="K26" s="438"/>
+      <c r="L26" s="438"/>
+      <c r="M26" s="438"/>
+      <c r="N26" s="438"/>
+      <c r="O26" s="438"/>
+      <c r="P26" s="438"/>
+      <c r="Q26" s="438"/>
+      <c r="R26" s="438"/>
+      <c r="S26" s="438"/>
+      <c r="T26" s="438"/>
+      <c r="U26" s="438"/>
+      <c r="V26" s="438"/>
+      <c r="W26" s="438"/>
+      <c r="X26" s="438"/>
+      <c r="Y26" s="438"/>
+      <c r="Z26" s="439"/>
+    </row>
+    <row r="27" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="437"/>
+      <c r="B27" s="438"/>
+      <c r="C27" s="438"/>
+      <c r="D27" s="438"/>
+      <c r="E27" s="438"/>
+      <c r="F27" s="438"/>
+      <c r="G27" s="438"/>
+      <c r="H27" s="438"/>
+      <c r="I27" s="438"/>
+      <c r="J27" s="438"/>
+      <c r="K27" s="438"/>
+      <c r="L27" s="438"/>
+      <c r="M27" s="438"/>
+      <c r="N27" s="438"/>
+      <c r="O27" s="438"/>
+      <c r="P27" s="438"/>
+      <c r="Q27" s="438"/>
+      <c r="R27" s="438"/>
+      <c r="S27" s="438"/>
+      <c r="T27" s="438"/>
+      <c r="U27" s="438"/>
+      <c r="V27" s="438"/>
+      <c r="W27" s="438"/>
+      <c r="X27" s="438"/>
+      <c r="Y27" s="438"/>
+      <c r="Z27" s="439"/>
+    </row>
+    <row r="28" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="437"/>
+      <c r="B28" s="438"/>
+      <c r="C28" s="438"/>
+      <c r="D28" s="438"/>
+      <c r="E28" s="438"/>
+      <c r="F28" s="438"/>
+      <c r="G28" s="438"/>
+      <c r="H28" s="438"/>
+      <c r="I28" s="438"/>
+      <c r="J28" s="438"/>
+      <c r="K28" s="438"/>
+      <c r="L28" s="438"/>
+      <c r="M28" s="438"/>
+      <c r="N28" s="438"/>
+      <c r="O28" s="438"/>
+      <c r="P28" s="438"/>
+      <c r="Q28" s="438"/>
+      <c r="R28" s="438"/>
+      <c r="S28" s="438"/>
+      <c r="T28" s="438"/>
+      <c r="U28" s="438"/>
+      <c r="V28" s="438"/>
+      <c r="W28" s="438"/>
+      <c r="X28" s="438"/>
+      <c r="Y28" s="438"/>
+      <c r="Z28" s="439"/>
+    </row>
+    <row r="29" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="437"/>
+      <c r="B29" s="438"/>
+      <c r="C29" s="438"/>
+      <c r="D29" s="438"/>
+      <c r="E29" s="438"/>
+      <c r="F29" s="438"/>
+      <c r="G29" s="438"/>
+      <c r="H29" s="438"/>
+      <c r="I29" s="438"/>
+      <c r="J29" s="438"/>
+      <c r="K29" s="438"/>
+      <c r="L29" s="438"/>
+      <c r="M29" s="438"/>
+      <c r="N29" s="438"/>
+      <c r="O29" s="438"/>
+      <c r="P29" s="438"/>
+      <c r="Q29" s="438"/>
+      <c r="R29" s="438"/>
+      <c r="S29" s="438"/>
+      <c r="T29" s="438"/>
+      <c r="U29" s="438"/>
+      <c r="V29" s="438"/>
+      <c r="W29" s="438"/>
+      <c r="X29" s="438"/>
+      <c r="Y29" s="438"/>
+      <c r="Z29" s="439"/>
+    </row>
+    <row r="30" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="437"/>
+      <c r="B30" s="438"/>
+      <c r="C30" s="438"/>
+      <c r="D30" s="438"/>
+      <c r="E30" s="438"/>
+      <c r="F30" s="438"/>
+      <c r="G30" s="438"/>
+      <c r="H30" s="438"/>
+      <c r="I30" s="438"/>
+      <c r="J30" s="438"/>
+      <c r="K30" s="438"/>
+      <c r="L30" s="438"/>
+      <c r="M30" s="438"/>
+      <c r="N30" s="438"/>
+      <c r="O30" s="438"/>
+      <c r="P30" s="438"/>
+      <c r="Q30" s="438"/>
+      <c r="R30" s="438"/>
+      <c r="S30" s="438"/>
+      <c r="T30" s="438"/>
+      <c r="U30" s="438"/>
+      <c r="V30" s="438"/>
+      <c r="W30" s="438"/>
+      <c r="X30" s="438"/>
+      <c r="Y30" s="438"/>
+      <c r="Z30" s="439"/>
+    </row>
+    <row r="31" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="437"/>
+      <c r="B31" s="438"/>
+      <c r="C31" s="438"/>
+      <c r="D31" s="438"/>
+      <c r="E31" s="438"/>
+      <c r="F31" s="438"/>
+      <c r="G31" s="438"/>
+      <c r="H31" s="438"/>
+      <c r="I31" s="438"/>
+      <c r="J31" s="438"/>
+      <c r="K31" s="438"/>
+      <c r="L31" s="438"/>
+      <c r="M31" s="438"/>
+      <c r="N31" s="438"/>
+      <c r="O31" s="438"/>
+      <c r="P31" s="438"/>
+      <c r="Q31" s="438"/>
+      <c r="R31" s="438"/>
+      <c r="S31" s="438"/>
+      <c r="T31" s="438"/>
+      <c r="U31" s="438"/>
+      <c r="V31" s="438"/>
+      <c r="W31" s="438"/>
+      <c r="X31" s="438"/>
+      <c r="Y31" s="438"/>
+      <c r="Z31" s="439"/>
+    </row>
+    <row r="32" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="437"/>
+      <c r="B32" s="438"/>
+      <c r="C32" s="438"/>
+      <c r="D32" s="438"/>
+      <c r="E32" s="438"/>
+      <c r="F32" s="438"/>
+      <c r="G32" s="438"/>
+      <c r="H32" s="438"/>
+      <c r="I32" s="438"/>
+      <c r="J32" s="438"/>
+      <c r="K32" s="438"/>
+      <c r="L32" s="438"/>
+      <c r="M32" s="438"/>
+      <c r="N32" s="438"/>
+      <c r="O32" s="438"/>
+      <c r="P32" s="438"/>
+      <c r="Q32" s="438"/>
+      <c r="R32" s="438"/>
+      <c r="S32" s="438"/>
+      <c r="T32" s="438"/>
+      <c r="U32" s="438"/>
+      <c r="V32" s="438"/>
+      <c r="W32" s="438"/>
+      <c r="X32" s="438"/>
+      <c r="Y32" s="438"/>
+      <c r="Z32" s="439"/>
+    </row>
+    <row r="33" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="437"/>
+      <c r="B33" s="438"/>
+      <c r="C33" s="438"/>
+      <c r="D33" s="438"/>
+      <c r="E33" s="438"/>
+      <c r="F33" s="438"/>
+      <c r="G33" s="438"/>
+      <c r="H33" s="438"/>
+      <c r="I33" s="438"/>
+      <c r="J33" s="438"/>
+      <c r="K33" s="438"/>
+      <c r="L33" s="438"/>
+      <c r="M33" s="438"/>
+      <c r="N33" s="438"/>
+      <c r="O33" s="438"/>
+      <c r="P33" s="438"/>
+      <c r="Q33" s="438"/>
+      <c r="R33" s="438"/>
+      <c r="S33" s="438"/>
+      <c r="T33" s="438"/>
+      <c r="U33" s="438"/>
+      <c r="V33" s="438"/>
+      <c r="W33" s="438"/>
+      <c r="X33" s="438"/>
+      <c r="Y33" s="438"/>
+      <c r="Z33" s="439"/>
+    </row>
+    <row r="34" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="437"/>
+      <c r="B34" s="438"/>
+      <c r="C34" s="438"/>
+      <c r="D34" s="438"/>
+      <c r="E34" s="438"/>
+      <c r="F34" s="438"/>
+      <c r="G34" s="438"/>
+      <c r="H34" s="438"/>
+      <c r="I34" s="438"/>
+      <c r="J34" s="438"/>
+      <c r="K34" s="438"/>
+      <c r="L34" s="438"/>
+      <c r="M34" s="438"/>
+      <c r="N34" s="438"/>
+      <c r="O34" s="438"/>
+      <c r="P34" s="438"/>
+      <c r="Q34" s="438"/>
+      <c r="R34" s="438"/>
+      <c r="S34" s="438"/>
+      <c r="T34" s="438"/>
+      <c r="U34" s="438"/>
+      <c r="V34" s="438"/>
+      <c r="W34" s="438"/>
+      <c r="X34" s="438"/>
+      <c r="Y34" s="438"/>
+      <c r="Z34" s="439"/>
+    </row>
+    <row r="35" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="437"/>
+      <c r="B35" s="438"/>
+      <c r="C35" s="438"/>
+      <c r="D35" s="438"/>
+      <c r="E35" s="438"/>
+      <c r="F35" s="438"/>
+      <c r="G35" s="438"/>
+      <c r="H35" s="438"/>
+      <c r="I35" s="438"/>
+      <c r="J35" s="438"/>
+      <c r="K35" s="438"/>
+      <c r="L35" s="438"/>
+      <c r="M35" s="438"/>
+      <c r="N35" s="438"/>
+      <c r="O35" s="438"/>
+      <c r="P35" s="438"/>
+      <c r="Q35" s="438"/>
+      <c r="R35" s="438"/>
+      <c r="S35" s="438"/>
+      <c r="T35" s="438"/>
+      <c r="U35" s="438"/>
+      <c r="V35" s="438"/>
+      <c r="W35" s="438"/>
+      <c r="X35" s="438"/>
+      <c r="Y35" s="438"/>
+      <c r="Z35" s="439"/>
+    </row>
+    <row r="36" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="437"/>
+      <c r="B36" s="438"/>
+      <c r="C36" s="438"/>
+      <c r="D36" s="438"/>
+      <c r="E36" s="438"/>
+      <c r="F36" s="438"/>
+      <c r="G36" s="438"/>
+      <c r="H36" s="438"/>
+      <c r="I36" s="438"/>
+      <c r="J36" s="438"/>
+      <c r="K36" s="438"/>
+      <c r="L36" s="438"/>
+      <c r="M36" s="438"/>
+      <c r="N36" s="438"/>
+      <c r="O36" s="438"/>
+      <c r="P36" s="438"/>
+      <c r="Q36" s="438"/>
+      <c r="R36" s="438"/>
+      <c r="S36" s="438"/>
+      <c r="T36" s="438"/>
+      <c r="U36" s="438"/>
+      <c r="V36" s="438"/>
+      <c r="W36" s="438"/>
+      <c r="X36" s="438"/>
+      <c r="Y36" s="438"/>
+      <c r="Z36" s="439"/>
+    </row>
+    <row r="37" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="437"/>
+      <c r="B37" s="438"/>
+      <c r="C37" s="438"/>
+      <c r="D37" s="438"/>
+      <c r="E37" s="438"/>
+      <c r="F37" s="438"/>
+      <c r="G37" s="438"/>
+      <c r="H37" s="438"/>
+      <c r="I37" s="438"/>
+      <c r="J37" s="438"/>
+      <c r="K37" s="438"/>
+      <c r="L37" s="438"/>
+      <c r="M37" s="438"/>
+      <c r="N37" s="438"/>
+      <c r="O37" s="438"/>
+      <c r="P37" s="438"/>
+      <c r="Q37" s="438"/>
+      <c r="R37" s="438"/>
+      <c r="S37" s="438"/>
+      <c r="T37" s="438"/>
+      <c r="U37" s="438"/>
+      <c r="V37" s="438"/>
+      <c r="W37" s="438"/>
+      <c r="X37" s="438"/>
+      <c r="Y37" s="438"/>
+      <c r="Z37" s="439"/>
+    </row>
+    <row r="38" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="437"/>
+      <c r="B38" s="438"/>
+      <c r="C38" s="438"/>
+      <c r="D38" s="438"/>
+      <c r="E38" s="438"/>
+      <c r="F38" s="438"/>
+      <c r="G38" s="438"/>
+      <c r="H38" s="438"/>
+      <c r="I38" s="438"/>
+      <c r="J38" s="438"/>
+      <c r="K38" s="438"/>
+      <c r="L38" s="438"/>
+      <c r="M38" s="438"/>
+      <c r="N38" s="438"/>
+      <c r="O38" s="438"/>
+      <c r="P38" s="438"/>
+      <c r="Q38" s="438"/>
+      <c r="R38" s="438"/>
+      <c r="S38" s="438"/>
+      <c r="T38" s="438"/>
+      <c r="U38" s="438"/>
+      <c r="V38" s="438"/>
+      <c r="W38" s="438"/>
+      <c r="X38" s="438"/>
+      <c r="Y38" s="438"/>
+      <c r="Z38" s="439"/>
+    </row>
+    <row r="39" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="437"/>
+      <c r="B39" s="438"/>
+      <c r="C39" s="438"/>
+      <c r="D39" s="438"/>
+      <c r="E39" s="438"/>
+      <c r="F39" s="438"/>
+      <c r="G39" s="438"/>
+      <c r="H39" s="438"/>
+      <c r="I39" s="438"/>
+      <c r="J39" s="438"/>
+      <c r="K39" s="438"/>
+      <c r="L39" s="438"/>
+      <c r="M39" s="438"/>
+      <c r="N39" s="438"/>
+      <c r="O39" s="438"/>
+      <c r="P39" s="438"/>
+      <c r="Q39" s="438"/>
+      <c r="R39" s="438"/>
+      <c r="S39" s="438"/>
+      <c r="T39" s="438"/>
+      <c r="U39" s="438"/>
+      <c r="V39" s="438"/>
+      <c r="W39" s="438"/>
+      <c r="X39" s="438"/>
+      <c r="Y39" s="438"/>
+      <c r="Z39" s="439"/>
+    </row>
+    <row r="40" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="437"/>
+      <c r="B40" s="438"/>
+      <c r="C40" s="438"/>
+      <c r="D40" s="438"/>
+      <c r="E40" s="438"/>
+      <c r="F40" s="438"/>
+      <c r="G40" s="438"/>
+      <c r="H40" s="438"/>
+      <c r="I40" s="438"/>
+      <c r="J40" s="438"/>
+      <c r="K40" s="438"/>
+      <c r="L40" s="438"/>
+      <c r="M40" s="438"/>
+      <c r="N40" s="438"/>
+      <c r="O40" s="438"/>
+      <c r="P40" s="438"/>
+      <c r="Q40" s="438"/>
+      <c r="R40" s="438"/>
+      <c r="S40" s="438"/>
+      <c r="T40" s="438"/>
+      <c r="U40" s="438"/>
+      <c r="V40" s="438"/>
+      <c r="W40" s="438"/>
+      <c r="X40" s="438"/>
+      <c r="Y40" s="438"/>
+      <c r="Z40" s="439"/>
+    </row>
+    <row r="41" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="437"/>
+      <c r="B41" s="438"/>
+      <c r="C41" s="438"/>
+      <c r="D41" s="438"/>
+      <c r="E41" s="438"/>
+      <c r="F41" s="438"/>
+      <c r="G41" s="438"/>
+      <c r="H41" s="438"/>
+      <c r="I41" s="438"/>
+      <c r="J41" s="438"/>
+      <c r="K41" s="438"/>
+      <c r="L41" s="438"/>
+      <c r="M41" s="438"/>
+      <c r="N41" s="438"/>
+      <c r="O41" s="438"/>
+      <c r="P41" s="438"/>
+      <c r="Q41" s="438"/>
+      <c r="R41" s="438"/>
+      <c r="S41" s="438"/>
+      <c r="T41" s="438"/>
+      <c r="U41" s="438"/>
+      <c r="V41" s="438"/>
+      <c r="W41" s="438"/>
+      <c r="X41" s="438"/>
+      <c r="Y41" s="438"/>
+      <c r="Z41" s="439"/>
+    </row>
+    <row r="42" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="437"/>
+      <c r="B42" s="438"/>
+      <c r="C42" s="438"/>
+      <c r="D42" s="438"/>
+      <c r="E42" s="438"/>
+      <c r="F42" s="438"/>
+      <c r="G42" s="438"/>
+      <c r="H42" s="438"/>
+      <c r="I42" s="438"/>
+      <c r="J42" s="438"/>
+      <c r="K42" s="438"/>
+      <c r="L42" s="438"/>
+      <c r="M42" s="438"/>
+      <c r="N42" s="438"/>
+      <c r="O42" s="438"/>
+      <c r="P42" s="438"/>
+      <c r="Q42" s="438"/>
+      <c r="R42" s="438"/>
+      <c r="S42" s="438"/>
+      <c r="T42" s="438"/>
+      <c r="U42" s="438"/>
+      <c r="V42" s="438"/>
+      <c r="W42" s="438"/>
+      <c r="X42" s="438"/>
+      <c r="Y42" s="438"/>
+      <c r="Z42" s="439"/>
+    </row>
+    <row r="43" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="437"/>
+      <c r="B43" s="438"/>
+      <c r="C43" s="438"/>
+      <c r="D43" s="438"/>
+      <c r="E43" s="438"/>
+      <c r="F43" s="438"/>
+      <c r="G43" s="438"/>
+      <c r="H43" s="438"/>
+      <c r="I43" s="438"/>
+      <c r="J43" s="438"/>
+      <c r="K43" s="438"/>
+      <c r="L43" s="438"/>
+      <c r="M43" s="438"/>
+      <c r="N43" s="438"/>
+      <c r="O43" s="438"/>
+      <c r="P43" s="438"/>
+      <c r="Q43" s="438"/>
+      <c r="R43" s="438"/>
+      <c r="S43" s="438"/>
+      <c r="T43" s="438"/>
+      <c r="U43" s="438"/>
+      <c r="V43" s="438"/>
+      <c r="W43" s="438"/>
+      <c r="X43" s="438"/>
+      <c r="Y43" s="438"/>
+      <c r="Z43" s="439"/>
+    </row>
+    <row r="44" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="437"/>
+      <c r="B44" s="438"/>
+      <c r="C44" s="438"/>
+      <c r="D44" s="438"/>
+      <c r="E44" s="438"/>
+      <c r="F44" s="438"/>
+      <c r="G44" s="438"/>
+      <c r="H44" s="438"/>
+      <c r="I44" s="438"/>
+      <c r="J44" s="438"/>
+      <c r="K44" s="438"/>
+      <c r="L44" s="438"/>
+      <c r="M44" s="438"/>
+      <c r="N44" s="438"/>
+      <c r="O44" s="438"/>
+      <c r="P44" s="438"/>
+      <c r="Q44" s="438"/>
+      <c r="R44" s="438"/>
+      <c r="S44" s="438"/>
+      <c r="T44" s="438"/>
+      <c r="U44" s="438"/>
+      <c r="V44" s="438"/>
+      <c r="W44" s="438"/>
+      <c r="X44" s="438"/>
+      <c r="Y44" s="438"/>
+      <c r="Z44" s="439"/>
+    </row>
+    <row r="45" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="437"/>
+      <c r="B45" s="438"/>
+      <c r="C45" s="438"/>
+      <c r="D45" s="438"/>
+      <c r="E45" s="438"/>
+      <c r="F45" s="438"/>
+      <c r="G45" s="438"/>
+      <c r="H45" s="438"/>
+      <c r="I45" s="438"/>
+      <c r="J45" s="438"/>
+      <c r="K45" s="438"/>
+      <c r="L45" s="438"/>
+      <c r="M45" s="438"/>
+      <c r="N45" s="438"/>
+      <c r="O45" s="438"/>
+      <c r="P45" s="438"/>
+      <c r="Q45" s="438"/>
+      <c r="R45" s="438"/>
+      <c r="S45" s="438"/>
+      <c r="T45" s="438"/>
+      <c r="U45" s="438"/>
+      <c r="V45" s="438"/>
+      <c r="W45" s="438"/>
+      <c r="X45" s="438"/>
+      <c r="Y45" s="438"/>
+      <c r="Z45" s="439"/>
+    </row>
+    <row r="46" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="437"/>
+      <c r="B46" s="438"/>
+      <c r="C46" s="438"/>
+      <c r="D46" s="438"/>
+      <c r="E46" s="438"/>
+      <c r="F46" s="438"/>
+      <c r="G46" s="438"/>
+      <c r="H46" s="438"/>
+      <c r="I46" s="438"/>
+      <c r="J46" s="438"/>
+      <c r="K46" s="438"/>
+      <c r="L46" s="438"/>
+      <c r="M46" s="438"/>
+      <c r="N46" s="438"/>
+      <c r="O46" s="438"/>
+      <c r="P46" s="438"/>
+      <c r="Q46" s="438"/>
+      <c r="R46" s="438"/>
+      <c r="S46" s="438"/>
+      <c r="T46" s="438"/>
+      <c r="U46" s="438"/>
+      <c r="V46" s="438"/>
+      <c r="W46" s="438"/>
+      <c r="X46" s="438"/>
+      <c r="Y46" s="438"/>
+      <c r="Z46" s="439"/>
+    </row>
+    <row r="47" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="437"/>
+      <c r="B47" s="438"/>
+      <c r="C47" s="438"/>
+      <c r="D47" s="438"/>
+      <c r="E47" s="438"/>
+      <c r="F47" s="438"/>
+      <c r="G47" s="438"/>
+      <c r="H47" s="438"/>
+      <c r="I47" s="438"/>
+      <c r="J47" s="438"/>
+      <c r="K47" s="438"/>
+      <c r="L47" s="438"/>
+      <c r="M47" s="438"/>
+      <c r="N47" s="438"/>
+      <c r="O47" s="438"/>
+      <c r="P47" s="438"/>
+      <c r="Q47" s="438"/>
+      <c r="R47" s="438"/>
+      <c r="S47" s="438"/>
+      <c r="T47" s="438"/>
+      <c r="U47" s="438"/>
+      <c r="V47" s="438"/>
+      <c r="W47" s="438"/>
+      <c r="X47" s="438"/>
+      <c r="Y47" s="438"/>
+      <c r="Z47" s="439"/>
+    </row>
+    <row r="48" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="437"/>
+      <c r="B48" s="438"/>
+      <c r="C48" s="438"/>
+      <c r="D48" s="438"/>
+      <c r="E48" s="438"/>
+      <c r="F48" s="438"/>
+      <c r="G48" s="438"/>
+      <c r="H48" s="438"/>
+      <c r="I48" s="438"/>
+      <c r="J48" s="438"/>
+      <c r="K48" s="438"/>
+      <c r="L48" s="438"/>
+      <c r="M48" s="438"/>
+      <c r="N48" s="438"/>
+      <c r="O48" s="438"/>
+      <c r="P48" s="438"/>
+      <c r="Q48" s="438"/>
+      <c r="R48" s="438"/>
+      <c r="S48" s="438"/>
+      <c r="T48" s="438"/>
+      <c r="U48" s="438"/>
+      <c r="V48" s="438"/>
+      <c r="W48" s="438"/>
+      <c r="X48" s="438"/>
+      <c r="Y48" s="438"/>
+      <c r="Z48" s="439"/>
+    </row>
+    <row r="49" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="437"/>
+      <c r="B49" s="438"/>
+      <c r="C49" s="438"/>
+      <c r="D49" s="438"/>
+      <c r="E49" s="438"/>
+      <c r="F49" s="438"/>
+      <c r="G49" s="438"/>
+      <c r="H49" s="438"/>
+      <c r="I49" s="438"/>
+      <c r="J49" s="438"/>
+      <c r="K49" s="438"/>
+      <c r="L49" s="438"/>
+      <c r="M49" s="438"/>
+      <c r="N49" s="438"/>
+      <c r="O49" s="438"/>
+      <c r="P49" s="438"/>
+      <c r="Q49" s="438"/>
+      <c r="R49" s="438"/>
+      <c r="S49" s="438"/>
+      <c r="T49" s="438"/>
+      <c r="U49" s="438"/>
+      <c r="V49" s="438"/>
+      <c r="W49" s="438"/>
+      <c r="X49" s="438"/>
+      <c r="Y49" s="438"/>
+      <c r="Z49" s="439"/>
+    </row>
+    <row r="50" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="437"/>
+      <c r="B50" s="438"/>
+      <c r="C50" s="438"/>
+      <c r="D50" s="438"/>
+      <c r="E50" s="438"/>
+      <c r="F50" s="438"/>
+      <c r="G50" s="438"/>
+      <c r="H50" s="438"/>
+      <c r="I50" s="438"/>
+      <c r="J50" s="438"/>
+      <c r="K50" s="438"/>
+      <c r="L50" s="438"/>
+      <c r="M50" s="438"/>
+      <c r="N50" s="438"/>
+      <c r="O50" s="438"/>
+      <c r="P50" s="438"/>
+      <c r="Q50" s="438"/>
+      <c r="R50" s="438"/>
+      <c r="S50" s="438"/>
+      <c r="T50" s="438"/>
+      <c r="U50" s="438"/>
+      <c r="V50" s="438"/>
+      <c r="W50" s="438"/>
+      <c r="X50" s="438"/>
+      <c r="Y50" s="438"/>
+      <c r="Z50" s="439"/>
+    </row>
+    <row r="51" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="437"/>
+      <c r="B51" s="438"/>
+      <c r="C51" s="438"/>
+      <c r="D51" s="438"/>
+      <c r="E51" s="438"/>
+      <c r="F51" s="438"/>
+      <c r="G51" s="438"/>
+      <c r="H51" s="438"/>
+      <c r="I51" s="438"/>
+      <c r="J51" s="438"/>
+      <c r="K51" s="438"/>
+      <c r="L51" s="438"/>
+      <c r="M51" s="438"/>
+      <c r="N51" s="438"/>
+      <c r="O51" s="438"/>
+      <c r="P51" s="438"/>
+      <c r="Q51" s="438"/>
+      <c r="R51" s="438"/>
+      <c r="S51" s="438"/>
+      <c r="T51" s="438"/>
+      <c r="U51" s="438"/>
+      <c r="V51" s="438"/>
+      <c r="W51" s="438"/>
+      <c r="X51" s="438"/>
+      <c r="Y51" s="438"/>
+      <c r="Z51" s="439"/>
+    </row>
+    <row r="52" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="437"/>
+      <c r="B52" s="438"/>
+      <c r="C52" s="438"/>
+      <c r="D52" s="438"/>
+      <c r="E52" s="438"/>
+      <c r="F52" s="438"/>
+      <c r="G52" s="438"/>
+      <c r="H52" s="438"/>
+      <c r="I52" s="438"/>
+      <c r="J52" s="438"/>
+      <c r="K52" s="438"/>
+      <c r="L52" s="438"/>
+      <c r="M52" s="438"/>
+      <c r="N52" s="438"/>
+      <c r="O52" s="438"/>
+      <c r="P52" s="438"/>
+      <c r="Q52" s="438"/>
+      <c r="R52" s="438"/>
+      <c r="S52" s="438"/>
+      <c r="T52" s="438"/>
+      <c r="U52" s="438"/>
+      <c r="V52" s="438"/>
+      <c r="W52" s="438"/>
+      <c r="X52" s="438"/>
+      <c r="Y52" s="438"/>
+      <c r="Z52" s="439"/>
+    </row>
+    <row r="53" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="437"/>
+      <c r="B53" s="438"/>
+      <c r="C53" s="438"/>
+      <c r="D53" s="438"/>
+      <c r="E53" s="438"/>
+      <c r="F53" s="438"/>
+      <c r="G53" s="438"/>
+      <c r="H53" s="438"/>
+      <c r="I53" s="438"/>
+      <c r="J53" s="438"/>
+      <c r="K53" s="438"/>
+      <c r="L53" s="438"/>
+      <c r="M53" s="438"/>
+      <c r="N53" s="438"/>
+      <c r="O53" s="438"/>
+      <c r="P53" s="438"/>
+      <c r="Q53" s="438"/>
+      <c r="R53" s="438"/>
+      <c r="S53" s="438"/>
+      <c r="T53" s="438"/>
+      <c r="U53" s="438"/>
+      <c r="V53" s="438"/>
+      <c r="W53" s="438"/>
+      <c r="X53" s="438"/>
+      <c r="Y53" s="438"/>
+      <c r="Z53" s="439"/>
+    </row>
+    <row r="54" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="437"/>
+      <c r="B54" s="438"/>
+      <c r="C54" s="438"/>
+      <c r="D54" s="438"/>
+      <c r="E54" s="438"/>
+      <c r="F54" s="438"/>
+      <c r="G54" s="438"/>
+      <c r="H54" s="438"/>
+      <c r="I54" s="438"/>
+      <c r="J54" s="438"/>
+      <c r="K54" s="438"/>
+      <c r="L54" s="438"/>
+      <c r="M54" s="438"/>
+      <c r="N54" s="438"/>
+      <c r="O54" s="438"/>
+      <c r="P54" s="438"/>
+      <c r="Q54" s="438"/>
+      <c r="R54" s="438"/>
+      <c r="S54" s="438"/>
+      <c r="T54" s="438"/>
+      <c r="U54" s="438"/>
+      <c r="V54" s="438"/>
+      <c r="W54" s="438"/>
+      <c r="X54" s="438"/>
+      <c r="Y54" s="438"/>
+      <c r="Z54" s="439"/>
+    </row>
+    <row r="55" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="437"/>
+      <c r="B55" s="438"/>
+      <c r="C55" s="438"/>
+      <c r="D55" s="438"/>
+      <c r="E55" s="438"/>
+      <c r="F55" s="438"/>
+      <c r="G55" s="438"/>
+      <c r="H55" s="438"/>
+      <c r="I55" s="438"/>
+      <c r="J55" s="438"/>
+      <c r="K55" s="438"/>
+      <c r="L55" s="438"/>
+      <c r="M55" s="438"/>
+      <c r="N55" s="438"/>
+      <c r="O55" s="438"/>
+      <c r="P55" s="438"/>
+      <c r="Q55" s="438"/>
+      <c r="R55" s="438"/>
+      <c r="S55" s="438"/>
+      <c r="T55" s="438"/>
+      <c r="U55" s="438"/>
+      <c r="V55" s="438"/>
+      <c r="W55" s="438"/>
+      <c r="X55" s="438"/>
+      <c r="Y55" s="438"/>
+      <c r="Z55" s="439"/>
+    </row>
+    <row r="56" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="437"/>
+      <c r="B56" s="438"/>
+      <c r="C56" s="438"/>
+      <c r="D56" s="438"/>
+      <c r="E56" s="438"/>
+      <c r="F56" s="438"/>
+      <c r="G56" s="438"/>
+      <c r="H56" s="438"/>
+      <c r="I56" s="438"/>
+      <c r="J56" s="438"/>
+      <c r="K56" s="438"/>
+      <c r="L56" s="438"/>
+      <c r="M56" s="438"/>
+      <c r="N56" s="438"/>
+      <c r="O56" s="438"/>
+      <c r="P56" s="438"/>
+      <c r="Q56" s="438"/>
+      <c r="R56" s="438"/>
+      <c r="S56" s="438"/>
+      <c r="T56" s="438"/>
+      <c r="U56" s="438"/>
+      <c r="V56" s="438"/>
+      <c r="W56" s="438"/>
+      <c r="X56" s="438"/>
+      <c r="Y56" s="438"/>
+      <c r="Z56" s="439"/>
+    </row>
+    <row r="57" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="171" t="s">
+        <v>126</v>
+      </c>
+      <c r="B57" s="380"/>
+      <c r="C57" s="381"/>
+      <c r="D57" s="382"/>
+      <c r="E57" s="382"/>
+      <c r="F57" s="382"/>
+      <c r="G57" s="382"/>
+      <c r="H57" s="382"/>
+      <c r="I57" s="382"/>
+      <c r="J57" s="171" t="s">
+        <v>141</v>
+      </c>
+      <c r="K57" s="380"/>
+      <c r="L57" s="381"/>
+      <c r="M57" s="382"/>
+      <c r="N57" s="382"/>
+      <c r="O57" s="382"/>
+      <c r="P57" s="382"/>
+      <c r="Q57" s="382"/>
+      <c r="R57" s="382"/>
+      <c r="S57" s="158"/>
+      <c r="T57" s="385"/>
+      <c r="U57" s="385"/>
+      <c r="V57" s="385"/>
+      <c r="W57" s="385"/>
+      <c r="X57" s="385"/>
+      <c r="Y57" s="385"/>
+      <c r="Z57" s="386"/>
+    </row>
+    <row r="58" spans="1:26" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="380"/>
+      <c r="B58" s="380"/>
+      <c r="C58" s="382"/>
+      <c r="D58" s="382"/>
+      <c r="E58" s="382"/>
+      <c r="F58" s="382"/>
+      <c r="G58" s="382"/>
+      <c r="H58" s="382"/>
+      <c r="I58" s="382"/>
+      <c r="J58" s="380"/>
+      <c r="K58" s="380"/>
+      <c r="L58" s="382"/>
+      <c r="M58" s="382"/>
+      <c r="N58" s="382"/>
+      <c r="O58" s="382"/>
+      <c r="P58" s="382"/>
+      <c r="Q58" s="382"/>
+      <c r="R58" s="382"/>
+      <c r="S58" s="387"/>
+      <c r="T58" s="388"/>
+      <c r="U58" s="388"/>
+      <c r="V58" s="388"/>
+      <c r="W58" s="388"/>
+      <c r="X58" s="388"/>
+      <c r="Y58" s="388"/>
+      <c r="Z58" s="389"/>
+    </row>
+    <row r="59" spans="1:26" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="380"/>
+      <c r="B59" s="380"/>
+      <c r="C59" s="382"/>
+      <c r="D59" s="382"/>
+      <c r="E59" s="382"/>
+      <c r="F59" s="382"/>
+      <c r="G59" s="382"/>
+      <c r="H59" s="382"/>
+      <c r="I59" s="382"/>
+      <c r="J59" s="380"/>
+      <c r="K59" s="380"/>
+      <c r="L59" s="382"/>
+      <c r="M59" s="382"/>
+      <c r="N59" s="382"/>
+      <c r="O59" s="382"/>
+      <c r="P59" s="382"/>
+      <c r="Q59" s="382"/>
+      <c r="R59" s="382"/>
+      <c r="S59" s="390"/>
+      <c r="T59" s="391"/>
+      <c r="U59" s="391"/>
+      <c r="V59" s="391"/>
+      <c r="W59" s="391"/>
+      <c r="X59" s="391"/>
+      <c r="Y59" s="391"/>
+      <c r="Z59" s="392"/>
+    </row>
+    <row r="60" spans="1:26" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="B60" s="121"/>
+      <c r="C60" s="383"/>
+      <c r="D60" s="383"/>
+      <c r="E60" s="383"/>
+      <c r="F60" s="383"/>
+      <c r="G60" s="383"/>
+      <c r="H60" s="383"/>
+      <c r="I60" s="383"/>
+      <c r="J60" s="383"/>
+      <c r="K60" s="383"/>
+      <c r="L60" s="383"/>
+      <c r="M60" s="383"/>
+      <c r="N60" s="383"/>
+      <c r="O60" s="383"/>
+      <c r="P60" s="383"/>
+      <c r="Q60" s="383"/>
+      <c r="R60" s="383"/>
+      <c r="S60" s="383"/>
+      <c r="T60" s="383"/>
+      <c r="U60" s="383"/>
+      <c r="V60" s="383"/>
+      <c r="W60" s="383"/>
+      <c r="X60" s="383"/>
+      <c r="Y60" s="383"/>
+      <c r="Z60" s="383"/>
+    </row>
+    <row r="61" spans="1:26" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="121"/>
+      <c r="B61" s="121"/>
+      <c r="C61" s="383"/>
+      <c r="D61" s="383"/>
+      <c r="E61" s="383"/>
+      <c r="F61" s="383"/>
+      <c r="G61" s="383"/>
+      <c r="H61" s="383"/>
+      <c r="I61" s="383"/>
+      <c r="J61" s="383"/>
+      <c r="K61" s="383"/>
+      <c r="L61" s="383"/>
+      <c r="M61" s="383"/>
+      <c r="N61" s="383"/>
+      <c r="O61" s="383"/>
+      <c r="P61" s="383"/>
+      <c r="Q61" s="383"/>
+      <c r="R61" s="383"/>
+      <c r="S61" s="383"/>
+      <c r="T61" s="383"/>
+      <c r="U61" s="383"/>
+      <c r="V61" s="383"/>
+      <c r="W61" s="383"/>
+      <c r="X61" s="383"/>
+      <c r="Y61" s="383"/>
+      <c r="Z61" s="383"/>
+    </row>
+    <row r="62" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="380"/>
+      <c r="B62" s="380"/>
+      <c r="C62" s="384"/>
+      <c r="D62" s="384"/>
+      <c r="E62" s="384"/>
+      <c r="F62" s="384"/>
+      <c r="G62" s="384"/>
+      <c r="H62" s="384"/>
+      <c r="I62" s="384"/>
+      <c r="J62" s="384"/>
+      <c r="K62" s="384"/>
+      <c r="L62" s="384"/>
+      <c r="M62" s="384"/>
+      <c r="N62" s="384"/>
+      <c r="O62" s="384"/>
+      <c r="P62" s="384"/>
+      <c r="Q62" s="384"/>
+      <c r="R62" s="384"/>
+      <c r="S62" s="384"/>
+      <c r="T62" s="384"/>
+      <c r="U62" s="384"/>
+      <c r="V62" s="384"/>
+      <c r="W62" s="384"/>
+      <c r="X62" s="384"/>
+      <c r="Y62" s="384"/>
+      <c r="Z62" s="384"/>
+    </row>
+    <row r="63" spans="1:26" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="380"/>
+      <c r="B63" s="380"/>
+      <c r="C63" s="384"/>
+      <c r="D63" s="384"/>
+      <c r="E63" s="384"/>
+      <c r="F63" s="384"/>
+      <c r="G63" s="384"/>
+      <c r="H63" s="384"/>
+      <c r="I63" s="384"/>
+      <c r="J63" s="384"/>
+      <c r="K63" s="384"/>
+      <c r="L63" s="384"/>
+      <c r="M63" s="384"/>
+      <c r="N63" s="384"/>
+      <c r="O63" s="384"/>
+      <c r="P63" s="384"/>
+      <c r="Q63" s="384"/>
+      <c r="R63" s="384"/>
+      <c r="S63" s="384"/>
+      <c r="T63" s="384"/>
+      <c r="U63" s="384"/>
+      <c r="V63" s="384"/>
+      <c r="W63" s="384"/>
+      <c r="X63" s="384"/>
+      <c r="Y63" s="384"/>
+      <c r="Z63" s="384"/>
+    </row>
+    <row r="64" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="121" t="s">
+        <v>44</v>
+      </c>
+      <c r="B64" s="121"/>
+      <c r="C64" s="445" t="str">
+        <f>IF(Report!C55="","",Report!C55)</f>
+        <v/>
+      </c>
+      <c r="D64" s="393"/>
+      <c r="E64" s="393"/>
+      <c r="F64" s="394"/>
+      <c r="G64" s="394"/>
+      <c r="H64" s="394"/>
+      <c r="I64" s="395" t="s">
+        <v>43</v>
+      </c>
+      <c r="J64" s="395"/>
+      <c r="K64" s="395"/>
+      <c r="L64" s="395"/>
+      <c r="M64" s="446" t="str">
+        <f>IF(Report!R55="","",Report!R55)</f>
+        <v/>
+      </c>
+      <c r="N64" s="380"/>
+      <c r="O64" s="380"/>
+      <c r="P64" s="380"/>
+      <c r="Q64" s="380"/>
+      <c r="R64" s="380"/>
+      <c r="S64" s="380"/>
+      <c r="T64" s="380"/>
+      <c r="U64" s="396"/>
+      <c r="V64" s="396"/>
+      <c r="W64" s="396"/>
+      <c r="X64" s="396"/>
+      <c r="Y64" s="396"/>
+      <c r="Z64" s="396"/>
+    </row>
+    <row r="65" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="121"/>
+      <c r="B65" s="121"/>
+      <c r="C65" s="393"/>
+      <c r="D65" s="393"/>
+      <c r="E65" s="393"/>
+      <c r="F65" s="394"/>
+      <c r="G65" s="394"/>
+      <c r="H65" s="394"/>
+      <c r="I65" s="395"/>
+      <c r="J65" s="395"/>
+      <c r="K65" s="395"/>
+      <c r="L65" s="395"/>
+      <c r="M65" s="380"/>
+      <c r="N65" s="380"/>
+      <c r="O65" s="380"/>
+      <c r="P65" s="380"/>
+      <c r="Q65" s="380"/>
+      <c r="R65" s="380"/>
+      <c r="S65" s="380"/>
+      <c r="T65" s="380"/>
+      <c r="U65" s="396"/>
+      <c r="V65" s="396"/>
+      <c r="W65" s="396"/>
+      <c r="X65" s="396"/>
+      <c r="Y65" s="396"/>
+      <c r="Z65" s="396"/>
+    </row>
+    <row r="66" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A66" s="373" t="s">
+        <v>53</v>
+      </c>
+      <c r="B66" s="373"/>
+      <c r="C66" s="373"/>
+      <c r="D66" s="373"/>
+      <c r="E66" s="373"/>
+      <c r="F66" s="373"/>
+      <c r="G66" s="373"/>
+      <c r="H66" s="373"/>
+      <c r="I66" s="373"/>
+      <c r="J66" s="373"/>
+      <c r="K66" s="373"/>
+      <c r="L66" s="373"/>
+      <c r="M66" s="373"/>
+      <c r="N66" s="373"/>
+      <c r="O66" s="373"/>
+      <c r="P66" s="373"/>
+      <c r="Q66" s="373"/>
+      <c r="R66" s="373"/>
+      <c r="S66" s="373"/>
+      <c r="T66" s="373"/>
+      <c r="U66" s="373"/>
+      <c r="V66" s="373"/>
+      <c r="W66" s="373"/>
+      <c r="X66" s="373"/>
+      <c r="Y66" s="373"/>
+      <c r="Z66" s="373"/>
+    </row>
+  </sheetData>
+  <mergeCells count="38">
+    <mergeCell ref="A66:Z66"/>
+    <mergeCell ref="A60:B63"/>
+    <mergeCell ref="C60:Z63"/>
+    <mergeCell ref="A64:B65"/>
+    <mergeCell ref="C64:H65"/>
+    <mergeCell ref="I64:L65"/>
+    <mergeCell ref="M64:T65"/>
+    <mergeCell ref="U64:Z65"/>
+    <mergeCell ref="A12:Z56"/>
+    <mergeCell ref="A57:B59"/>
+    <mergeCell ref="C57:I59"/>
+    <mergeCell ref="J57:K59"/>
+    <mergeCell ref="L57:R59"/>
+    <mergeCell ref="S57:Z59"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:I11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L11:R11"/>
+    <mergeCell ref="S11:T11"/>
+    <mergeCell ref="U11:X11"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:Z8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:Z9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:Z10"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="V5:W5"/>
+    <mergeCell ref="X5:Z5"/>
+    <mergeCell ref="A6:Z6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:Z7"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="X1:Z1"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Z2"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.25" right="0.39" top="0.25" bottom="0.25" header="0.05" footer="0.25"/>
+  <pageSetup scale="68" orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;C
+Houston, Texas 77099 • Telephone 713-366-0700 • Fax 713-366-0701</oddFooter>
   </headerFooter>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>